<commit_message>
Mela management module added
</commit_message>
<xml_diff>
--- a/_data_list/BTS_List_MO.xlsx
+++ b/_data_list/BTS_List_MO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Telegram_Project\OrangeFlow_Dev\_data_list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC7DEC0D-E4D9-4DCF-8E2C-0587B1BA848C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E25F0497-B7C7-485F-9750-AD3409CD3350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,10 +16,21 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AA$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AB$36</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -28,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="806" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="842" uniqueCount="262">
   <si>
     <t>SITE ID</t>
   </si>
@@ -432,9 +443,6 @@
     <t>বরাগীরকান্দি, আদমপুর বাজার, অষ্টগ্রাম, কিশোরগঞ্জ</t>
   </si>
   <si>
-    <t>বরাগীরকান্দি আদমপুর বাজার</t>
-  </si>
-  <si>
     <t>Choudonto Poschimpara  Adompur   Aostogram Kishorgonj</t>
   </si>
   <si>
@@ -486,9 +494,6 @@
     <t>পূর্ব অষ্টগ্রাম (হাজী বাড়ি), অষ্টগ্রাম, কিশোরগঞ্জ</t>
   </si>
   <si>
-    <t>পূর্ব (হাজী বাড়ি)</t>
-  </si>
-  <si>
     <t>Savianagar, Astagram, Kishoreganj</t>
   </si>
   <si>
@@ -522,18 +527,12 @@
     <t>বরশীকুড়া বাদলা ইটনা কিশোরগঞ্জ</t>
   </si>
   <si>
-    <t xml:space="preserve">বরশীকুড়া বাদলা  </t>
-  </si>
-  <si>
     <t>Chandrapur, Neyamotpur, Karimganj, Kishoreganj</t>
   </si>
   <si>
     <t>চন্দ্রপুর, নেয়ামতপুর, করিমগঞ্জ, কিশোরগঞ্জ</t>
   </si>
   <si>
-    <t>চন্দ্রপুর নেয়ামতপুর করিমগঞ্জ</t>
-  </si>
-  <si>
     <t>Dhonpur Bazar,Itna,Kishoreganj</t>
   </si>
   <si>
@@ -712,6 +711,120 @@
   </si>
   <si>
     <t>Rural</t>
+  </si>
+  <si>
+    <t>SHORT ADDRESS BN</t>
+  </si>
+  <si>
+    <t>Abdullahpur</t>
+  </si>
+  <si>
+    <t>Ali Nagar</t>
+  </si>
+  <si>
+    <t>Austogram</t>
+  </si>
+  <si>
+    <t>Bangal Para</t>
+  </si>
+  <si>
+    <t>Boragirkandi</t>
+  </si>
+  <si>
+    <t>Mosjid Zam (Sonarhati)</t>
+  </si>
+  <si>
+    <t>Puba Kolapara</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Purba Astagram(Hazi Bari) </t>
+  </si>
+  <si>
+    <t>Savianagar</t>
+  </si>
+  <si>
+    <t>Elenjuri</t>
+  </si>
+  <si>
+    <t>Borohati</t>
+  </si>
+  <si>
+    <t>Chandrapur</t>
+  </si>
+  <si>
+    <t>Dhonpur Bazar</t>
+  </si>
+  <si>
+    <t>Joysiddi Bazar</t>
+  </si>
+  <si>
+    <t>Purbo Gram (Thakurhati)</t>
+  </si>
+  <si>
+    <t>Saidur Rahman Thakur</t>
+  </si>
+  <si>
+    <t>Dhaki Bazar</t>
+  </si>
+  <si>
+    <t>Ghagra Bazar</t>
+  </si>
+  <si>
+    <t>Girishpur</t>
+  </si>
+  <si>
+    <t>Gopdighi</t>
+  </si>
+  <si>
+    <t>Hemontoganj</t>
+  </si>
+  <si>
+    <t>Islampur</t>
+  </si>
+  <si>
+    <t>Kamalpur</t>
+  </si>
+  <si>
+    <t>Keowarjor Bazar</t>
+  </si>
+  <si>
+    <t>Katkhal Bazar</t>
+  </si>
+  <si>
+    <t>Mithamain Bazar</t>
+  </si>
+  <si>
+    <t>বরাগীরকান্দি</t>
+  </si>
+  <si>
+    <t>Choudonto Poschimpara </t>
+  </si>
+  <si>
+    <t>Kastol</t>
+  </si>
+  <si>
+    <t>Kolimpur  Abdullahpur</t>
+  </si>
+  <si>
+    <t>পূর্ব অষ্টগ্রাম (হাজী বাড়ি)</t>
+  </si>
+  <si>
+    <t>Borshikura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">বরশীকুড়া  </t>
+  </si>
+  <si>
+    <t>চন্দ্রপুর</t>
+  </si>
+  <si>
+    <t>Joyonshai Sohila</t>
+  </si>
+  <si>
+    <t>Panch Hat Khaliajuri</t>
+  </si>
+  <si>
+    <t>Dholai Gopdighi</t>
   </si>
 </sst>
 </file>
@@ -721,7 +834,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]d/mmm/yy;@"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -733,6 +846,12 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -770,7 +889,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -781,6 +900,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1083,7 +1205,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA36"/>
+  <dimension ref="A1:AB36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -1102,16 +1224,17 @@
     <col min="14" max="14" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="53.85546875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="49.28515625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="28.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="12" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="23" max="25" width="14" style="3" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="19" max="20" width="12" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="24" max="26" width="14" style="3" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="14.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1163,38 +1286,41 @@
       <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="S1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="2" t="s">
+      <c r="X1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>32</v>
       </c>
@@ -1244,38 +1370,41 @@
         <v>120</v>
       </c>
       <c r="Q2" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="R2" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="R2" s="4">
+      <c r="S2" s="4">
         <v>91.165599999999998</v>
       </c>
-      <c r="S2" s="4">
+      <c r="T2" s="4">
         <v>24.390899999999998</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="U2" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="V2" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="W2" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W2" s="5">
+      <c r="X2" s="5">
         <v>43253</v>
       </c>
-      <c r="X2" s="5"/>
-      <c r="Y2" s="5">
+      <c r="Y2" s="5"/>
+      <c r="Z2" s="5">
         <v>43901</v>
-      </c>
-      <c r="Z2" s="4" t="s">
-        <v>227</v>
       </c>
       <c r="AA2" s="4" t="s">
         <v>223</v>
       </c>
+      <c r="AB2" s="4" t="s">
+        <v>219</v>
+      </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>40</v>
       </c>
@@ -1325,38 +1454,41 @@
         <v>124</v>
       </c>
       <c r="Q3" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="R3" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="R3" s="4">
+      <c r="S3" s="4">
         <v>91.072388888888881</v>
       </c>
-      <c r="S3" s="4">
+      <c r="T3" s="4">
         <v>24.281583333333334</v>
       </c>
-      <c r="T3" s="4" t="s">
+      <c r="U3" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U3" s="4" t="s">
+      <c r="V3" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V3" s="4" t="s">
+      <c r="W3" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W3" s="5">
+      <c r="X3" s="5">
         <v>43300</v>
       </c>
-      <c r="X3" s="5"/>
-      <c r="Y3" s="5">
+      <c r="Y3" s="5"/>
+      <c r="Z3" s="5">
         <v>43856</v>
-      </c>
-      <c r="Z3" s="4" t="s">
-        <v>227</v>
       </c>
       <c r="AA3" s="4" t="s">
         <v>223</v>
       </c>
+      <c r="AB3" s="4" t="s">
+        <v>219</v>
+      </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>42</v>
       </c>
@@ -1406,38 +1538,41 @@
         <v>127</v>
       </c>
       <c r="Q4" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="R4" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="R4" s="4">
+      <c r="S4" s="4">
         <v>91.109660000000005</v>
       </c>
-      <c r="S4" s="4">
+      <c r="T4" s="4">
         <v>24.27758</v>
       </c>
-      <c r="T4" s="4" t="s">
+      <c r="U4" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U4" s="4" t="s">
+      <c r="V4" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V4" s="4" t="s">
+      <c r="W4" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W4" s="5">
+      <c r="X4" s="5">
         <v>39350</v>
       </c>
-      <c r="X4" s="5"/>
-      <c r="Y4" s="5">
+      <c r="Y4" s="5"/>
+      <c r="Z4" s="5">
         <v>43642</v>
       </c>
-      <c r="Z4" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="AA4" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
+      </c>
+      <c r="AB4" s="4" t="s">
+        <v>220</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>44</v>
       </c>
@@ -1487,38 +1622,41 @@
         <v>130</v>
       </c>
       <c r="Q5" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="R5" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="R5" s="4">
+      <c r="S5" s="4">
         <v>91.113200000000006</v>
       </c>
-      <c r="S5" s="4">
+      <c r="T5" s="4">
         <v>24.2441</v>
       </c>
-      <c r="T5" s="4" t="s">
+      <c r="U5" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U5" s="4" t="s">
+      <c r="V5" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V5" s="4" t="s">
+      <c r="W5" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W5" s="5">
+      <c r="X5" s="5">
         <v>42908</v>
       </c>
-      <c r="X5" s="5"/>
-      <c r="Y5" s="5">
+      <c r="Y5" s="5"/>
+      <c r="Z5" s="5">
         <v>43890</v>
-      </c>
-      <c r="Z5" s="4" t="s">
-        <v>227</v>
       </c>
       <c r="AA5" s="4" t="s">
         <v>223</v>
       </c>
+      <c r="AB5" s="4" t="s">
+        <v>219</v>
+      </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>46</v>
       </c>
@@ -1568,38 +1706,41 @@
         <v>133</v>
       </c>
       <c r="Q6" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="R6" s="4">
+        <v>229</v>
+      </c>
+      <c r="R6" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="S6" s="4">
         <v>91.2179</v>
       </c>
-      <c r="S6" s="4">
+      <c r="T6" s="4">
         <v>24.350580000000001</v>
       </c>
-      <c r="T6" s="4" t="s">
+      <c r="U6" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U6" s="4" t="s">
+      <c r="V6" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V6" s="4" t="s">
+      <c r="W6" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W6" s="5">
+      <c r="X6" s="5">
         <v>43708</v>
       </c>
-      <c r="X6" s="5"/>
-      <c r="Y6" s="5">
+      <c r="Y6" s="5"/>
+      <c r="Z6" s="5">
         <v>43858</v>
-      </c>
-      <c r="Z6" s="4" t="s">
-        <v>227</v>
       </c>
       <c r="AA6" s="4" t="s">
         <v>223</v>
       </c>
+      <c r="AB6" s="4" t="s">
+        <v>219</v>
+      </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>48</v>
       </c>
@@ -1643,44 +1784,47 @@
         <v>116</v>
       </c>
       <c r="O7" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="P7" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="P7" s="4" t="s">
+      <c r="Q7" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="R7" s="4" t="s">
         <v>136</v>
       </c>
-      <c r="Q7" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="R7" s="4">
+      <c r="S7" s="4">
         <v>91.152720000000002</v>
       </c>
-      <c r="S7" s="4">
+      <c r="T7" s="4">
         <v>24.333870000000001</v>
       </c>
-      <c r="T7" s="4" t="s">
+      <c r="U7" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U7" s="4" t="s">
+      <c r="V7" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V7" s="4" t="s">
+      <c r="W7" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W7" s="5">
+      <c r="X7" s="5">
         <v>44253</v>
       </c>
-      <c r="X7" s="5"/>
-      <c r="Y7" s="5">
+      <c r="Y7" s="5"/>
+      <c r="Z7" s="5">
         <v>44253</v>
-      </c>
-      <c r="Z7" s="4" t="s">
-        <v>227</v>
       </c>
       <c r="AA7" s="4" t="s">
         <v>223</v>
       </c>
+      <c r="AB7" s="4" t="s">
+        <v>219</v>
+      </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>50</v>
       </c>
@@ -1724,46 +1868,49 @@
         <v>116</v>
       </c>
       <c r="O8" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="P8" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="P8" s="4" t="s">
+      <c r="Q8" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="R8" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="Q8" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="R8" s="4">
+      <c r="S8" s="4">
         <v>91.082126000000002</v>
       </c>
-      <c r="S8" s="4">
+      <c r="T8" s="4">
         <v>24.288474999999998</v>
       </c>
-      <c r="T8" s="4" t="s">
+      <c r="U8" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U8" s="4" t="s">
+      <c r="V8" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V8" s="4" t="s">
+      <c r="W8" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W8" s="5">
+      <c r="X8" s="5">
         <v>44318</v>
       </c>
-      <c r="X8" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="Y8" s="5">
+      <c r="Y8" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="Z8" s="5">
         <v>44318</v>
-      </c>
-      <c r="Z8" s="4" t="s">
-        <v>227</v>
       </c>
       <c r="AA8" s="4" t="s">
         <v>223</v>
       </c>
+      <c r="AB8" s="4" t="s">
+        <v>219</v>
+      </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>52</v>
       </c>
@@ -1807,44 +1954,47 @@
         <v>116</v>
       </c>
       <c r="O9" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="P9" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="P9" s="4" t="s">
+      <c r="Q9" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="R9" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="Q9" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="R9" s="4">
+      <c r="S9" s="4">
         <v>91.182575</v>
       </c>
-      <c r="S9" s="4">
+      <c r="T9" s="4">
         <v>24.402118000000002</v>
       </c>
-      <c r="T9" s="4" t="s">
+      <c r="U9" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U9" s="4" t="s">
+      <c r="V9" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V9" s="4" t="s">
+      <c r="W9" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W9" s="5">
+      <c r="X9" s="5">
         <v>44251</v>
       </c>
-      <c r="X9" s="5"/>
-      <c r="Y9" s="5">
+      <c r="Y9" s="5"/>
+      <c r="Z9" s="5">
         <v>44251</v>
       </c>
-      <c r="Z9" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="AA9" s="4" t="s">
-        <v>225</v>
+        <v>223</v>
+      </c>
+      <c r="AB9" s="4" t="s">
+        <v>221</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>54</v>
       </c>
@@ -1888,46 +2038,49 @@
         <v>116</v>
       </c>
       <c r="O10" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="P10" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="P10" s="4" t="s">
+      <c r="Q10" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="R10" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="Q10" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="R10" s="4">
+      <c r="S10" s="4">
         <v>91.099395999999999</v>
       </c>
-      <c r="S10" s="4">
+      <c r="T10" s="4">
         <v>24.278690999999998</v>
       </c>
-      <c r="T10" s="4" t="s">
+      <c r="U10" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U10" s="4" t="s">
+      <c r="V10" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V10" s="4" t="s">
+      <c r="W10" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W10" s="5">
+      <c r="X10" s="5">
         <v>44346</v>
       </c>
-      <c r="X10" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="Y10" s="5">
+      <c r="Y10" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="Z10" s="5">
         <v>44346</v>
-      </c>
-      <c r="Z10" s="4" t="s">
-        <v>227</v>
       </c>
       <c r="AA10" s="4" t="s">
         <v>223</v>
       </c>
+      <c r="AB10" s="4" t="s">
+        <v>219</v>
+      </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>56</v>
       </c>
@@ -1971,46 +2124,49 @@
         <v>116</v>
       </c>
       <c r="O11" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="P11" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="P11" s="4" t="s">
+      <c r="Q11" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="R11" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="Q11" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="R11" s="4">
+      <c r="S11" s="4">
         <v>91.120186000000004</v>
       </c>
-      <c r="S11" s="4">
+      <c r="T11" s="4">
         <v>24.279910000000001</v>
       </c>
-      <c r="T11" s="4" t="s">
+      <c r="U11" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U11" s="4" t="s">
+      <c r="V11" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V11" s="4" t="s">
+      <c r="W11" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W11" s="5">
+      <c r="X11" s="5">
         <v>44396</v>
       </c>
-      <c r="X11" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="Y11" s="5">
+      <c r="Y11" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="Z11" s="5">
         <v>44396</v>
       </c>
-      <c r="Z11" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="AA11" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
+      </c>
+      <c r="AB11" s="4" t="s">
+        <v>220</v>
       </c>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>58</v>
       </c>
@@ -2054,44 +2210,47 @@
         <v>116</v>
       </c>
       <c r="O12" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="P12" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="P12" s="4" t="s">
-        <v>151</v>
-      </c>
       <c r="Q12" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="R12" s="4">
+        <v>232</v>
+      </c>
+      <c r="R12" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="S12" s="4">
         <v>91.134799999999998</v>
       </c>
-      <c r="S12" s="4">
+      <c r="T12" s="4">
         <v>24.277450000000002</v>
       </c>
-      <c r="T12" s="4" t="s">
+      <c r="U12" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U12" s="4" t="s">
+      <c r="V12" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V12" s="4" t="s">
+      <c r="W12" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W12" s="5">
+      <c r="X12" s="5">
         <v>39781</v>
       </c>
-      <c r="X12" s="5"/>
-      <c r="Y12" s="5">
+      <c r="Y12" s="5"/>
+      <c r="Z12" s="5">
         <v>43767</v>
       </c>
-      <c r="Z12" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="AA12" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
+      </c>
+      <c r="AB12" s="4" t="s">
+        <v>220</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>60</v>
       </c>
@@ -2135,44 +2294,47 @@
         <v>116</v>
       </c>
       <c r="O13" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="P13" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="Q13" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="R13" s="4" t="s">
         <v>153</v>
       </c>
-      <c r="P13" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="Q13" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="R13" s="4">
+      <c r="S13" s="4">
         <v>91.089190000000002</v>
       </c>
-      <c r="S13" s="4">
+      <c r="T13" s="4">
         <v>24.273790000000002</v>
       </c>
-      <c r="T13" s="4" t="s">
+      <c r="U13" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U13" s="4" t="s">
+      <c r="V13" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V13" s="4" t="s">
+      <c r="W13" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W13" s="5">
+      <c r="X13" s="5">
         <v>41298</v>
       </c>
-      <c r="X13" s="5"/>
-      <c r="Y13" s="5">
+      <c r="Y13" s="5"/>
+      <c r="Z13" s="5">
         <v>43767</v>
       </c>
-      <c r="Z13" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="AA13" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
+      </c>
+      <c r="AB13" s="4" t="s">
+        <v>220</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>62</v>
       </c>
@@ -2216,44 +2378,47 @@
         <v>116</v>
       </c>
       <c r="O14" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="P14" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="Q14" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="R14" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="P14" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q14" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="R14" s="4">
+      <c r="S14" s="4">
         <v>91.052520000000001</v>
       </c>
-      <c r="S14" s="4">
+      <c r="T14" s="4">
         <v>24.495280000000001</v>
       </c>
-      <c r="T14" s="4" t="s">
+      <c r="U14" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U14" s="4" t="s">
+      <c r="V14" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V14" s="4" t="s">
+      <c r="W14" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W14" s="5">
+      <c r="X14" s="5">
         <v>39953</v>
       </c>
-      <c r="X14" s="5"/>
-      <c r="Y14" s="5">
+      <c r="Y14" s="5"/>
+      <c r="Z14" s="5">
         <v>43767</v>
       </c>
-      <c r="Z14" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="AA14" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
+      </c>
+      <c r="AB14" s="4" t="s">
+        <v>220</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>66</v>
       </c>
@@ -2297,46 +2462,49 @@
         <v>116</v>
       </c>
       <c r="O15" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="P15" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="Q15" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="R15" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="P15" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="Q15" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="R15" s="4">
+      <c r="S15" s="4">
         <v>91.092200000000005</v>
       </c>
-      <c r="S15" s="4">
+      <c r="T15" s="4">
         <v>24.5244</v>
       </c>
-      <c r="T15" s="4" t="s">
+      <c r="U15" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U15" s="4" t="s">
+      <c r="V15" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V15" s="4" t="s">
+      <c r="W15" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W15" s="5">
+      <c r="X15" s="5">
         <v>44460</v>
       </c>
-      <c r="X15" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="Y15" s="5">
+      <c r="Y15" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="Z15" s="5">
         <v>44460</v>
       </c>
-      <c r="Z15" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="AA15" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
+      </c>
+      <c r="AB15" s="4" t="s">
+        <v>220</v>
       </c>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>68</v>
       </c>
@@ -2380,46 +2548,49 @@
         <v>116</v>
       </c>
       <c r="O16" s="4" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="P16" s="4" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="Q16" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="R16" s="4">
+        <v>256</v>
+      </c>
+      <c r="R16" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="S16" s="4">
         <v>91.014930000000007</v>
       </c>
-      <c r="S16" s="4">
+      <c r="T16" s="4">
         <v>24.560379999999999</v>
       </c>
-      <c r="T16" s="4" t="s">
+      <c r="U16" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U16" s="4" t="s">
+      <c r="V16" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V16" s="4" t="s">
+      <c r="W16" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W16" s="5">
+      <c r="X16" s="5">
         <v>44439</v>
       </c>
-      <c r="X16" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="Y16" s="5">
+      <c r="Y16" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="Z16" s="5">
         <v>44439</v>
-      </c>
-      <c r="Z16" s="4" t="s">
-        <v>227</v>
       </c>
       <c r="AA16" s="4" t="s">
         <v>223</v>
       </c>
+      <c r="AB16" s="4" t="s">
+        <v>219</v>
+      </c>
     </row>
-    <row r="17" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>70</v>
       </c>
@@ -2463,46 +2634,49 @@
         <v>116</v>
       </c>
       <c r="O17" s="4" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="P17" s="4" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="Q17" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="R17" s="4">
+        <v>236</v>
+      </c>
+      <c r="R17" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="S17" s="4">
         <v>90.954183</v>
       </c>
-      <c r="S17" s="4">
+      <c r="T17" s="4">
         <v>24.497088999999999</v>
       </c>
-      <c r="T17" s="4" t="s">
+      <c r="U17" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U17" s="4" t="s">
+      <c r="V17" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V17" s="4" t="s">
+      <c r="W17" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W17" s="5">
+      <c r="X17" s="5">
         <v>45365</v>
       </c>
-      <c r="X17" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="Y17" s="5">
+      <c r="Y17" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="Z17" s="5">
         <v>45365</v>
       </c>
-      <c r="Z17" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="AA17" s="4" t="s">
-        <v>225</v>
+        <v>223</v>
+      </c>
+      <c r="AB17" s="4" t="s">
+        <v>221</v>
       </c>
     </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>72</v>
       </c>
@@ -2546,44 +2720,47 @@
         <v>116</v>
       </c>
       <c r="O18" s="4" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P18" s="4" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="Q18" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="R18" s="4">
+        <v>237</v>
+      </c>
+      <c r="R18" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="S18" s="4">
         <v>91.131259999999997</v>
       </c>
-      <c r="S18" s="4">
+      <c r="T18" s="4">
         <v>24.601179999999999</v>
       </c>
-      <c r="T18" s="4" t="s">
+      <c r="U18" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U18" s="4" t="s">
+      <c r="V18" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V18" s="4" t="s">
+      <c r="W18" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W18" s="5">
+      <c r="X18" s="5">
         <v>42184</v>
       </c>
-      <c r="X18" s="5"/>
-      <c r="Y18" s="5">
+      <c r="Y18" s="5"/>
+      <c r="Z18" s="5">
         <v>44217</v>
       </c>
-      <c r="Z18" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="AA18" s="4" t="s">
-        <v>225</v>
+        <v>223</v>
+      </c>
+      <c r="AB18" s="4" t="s">
+        <v>221</v>
       </c>
     </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>74</v>
       </c>
@@ -2627,44 +2804,47 @@
         <v>116</v>
       </c>
       <c r="O19" s="4" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="P19" s="4" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="Q19" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="R19" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="R19" s="4">
+      <c r="S19" s="4">
         <v>91.086380000000005</v>
       </c>
-      <c r="S19" s="4">
+      <c r="T19" s="4">
         <v>24.528269999999999</v>
       </c>
-      <c r="T19" s="4" t="s">
+      <c r="U19" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U19" s="4" t="s">
+      <c r="V19" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V19" s="4" t="s">
+      <c r="W19" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W19" s="5">
+      <c r="X19" s="5">
         <v>40418</v>
       </c>
-      <c r="X19" s="5"/>
-      <c r="Y19" s="5">
+      <c r="Y19" s="5"/>
+      <c r="Z19" s="5">
         <v>43856</v>
       </c>
-      <c r="Z19" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="AA19" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
+      </c>
+      <c r="AB19" s="4" t="s">
+        <v>220</v>
       </c>
     </row>
-    <row r="20" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>76</v>
       </c>
@@ -2708,44 +2888,47 @@
         <v>116</v>
       </c>
       <c r="O20" s="4" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="P20" s="4" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="Q20" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="R20" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="R20" s="4">
+      <c r="S20" s="4">
         <v>90.980779999999996</v>
       </c>
-      <c r="S20" s="4">
+      <c r="T20" s="4">
         <v>24.58108</v>
       </c>
-      <c r="T20" s="4" t="s">
+      <c r="U20" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U20" s="4" t="s">
+      <c r="V20" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V20" s="4" t="s">
+      <c r="W20" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W20" s="5">
+      <c r="X20" s="5">
         <v>45181</v>
       </c>
-      <c r="X20" s="5"/>
-      <c r="Y20" s="5">
+      <c r="Y20" s="5"/>
+      <c r="Z20" s="5">
         <v>45181</v>
-      </c>
-      <c r="Z20" s="4" t="s">
-        <v>227</v>
       </c>
       <c r="AA20" s="4" t="s">
         <v>223</v>
       </c>
+      <c r="AB20" s="4" t="s">
+        <v>219</v>
+      </c>
     </row>
-    <row r="21" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>78</v>
       </c>
@@ -2789,46 +2972,49 @@
         <v>116</v>
       </c>
       <c r="O21" s="4" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="P21" s="4" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="Q21" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="R21" s="4">
+        <v>259</v>
+      </c>
+      <c r="R21" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="S21" s="4">
         <v>91.109348900000001</v>
       </c>
-      <c r="S21" s="4">
+      <c r="T21" s="4">
         <v>24.563555000000001</v>
       </c>
-      <c r="T21" s="4" t="s">
+      <c r="U21" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U21" s="4" t="s">
+      <c r="V21" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V21" s="4" t="s">
+      <c r="W21" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W21" s="5">
+      <c r="X21" s="5">
         <v>44651</v>
       </c>
-      <c r="X21" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="Y21" s="5">
+      <c r="Y21" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="Z21" s="5">
         <v>44651</v>
       </c>
-      <c r="Z21" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="AA21" s="4" t="s">
-        <v>225</v>
+        <v>223</v>
+      </c>
+      <c r="AB21" s="4" t="s">
+        <v>221</v>
       </c>
     </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
         <v>80</v>
       </c>
@@ -2872,44 +3058,47 @@
         <v>116</v>
       </c>
       <c r="O22" s="4" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="P22" s="4" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="Q22" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="R22" s="4">
+        <v>238</v>
+      </c>
+      <c r="R22" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="S22" s="4">
         <v>91.137420000000006</v>
       </c>
-      <c r="S22" s="4">
+      <c r="T22" s="4">
         <v>24.508600000000001</v>
       </c>
-      <c r="T22" s="4" t="s">
+      <c r="U22" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U22" s="4" t="s">
+      <c r="V22" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V22" s="4" t="s">
+      <c r="W22" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W22" s="5">
+      <c r="X22" s="5">
         <v>39950</v>
       </c>
-      <c r="X22" s="5"/>
-      <c r="Y22" s="5">
+      <c r="Y22" s="5"/>
+      <c r="Z22" s="5">
         <v>43782</v>
       </c>
-      <c r="Z22" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="AA22" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
+      </c>
+      <c r="AB22" s="4" t="s">
+        <v>220</v>
       </c>
     </row>
-    <row r="23" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>82</v>
       </c>
@@ -2953,44 +3142,47 @@
         <v>116</v>
       </c>
       <c r="O23" s="4" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="P23" s="4" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="Q23" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="R23" s="4">
+        <v>239</v>
+      </c>
+      <c r="R23" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="S23" s="4">
         <v>91.109889999999993</v>
       </c>
-      <c r="S23" s="4">
+      <c r="T23" s="4">
         <v>24.533729999999998</v>
       </c>
-      <c r="T23" s="4" t="s">
+      <c r="U23" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U23" s="4" t="s">
+      <c r="V23" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V23" s="4" t="s">
+      <c r="W23" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W23" s="5">
+      <c r="X23" s="5">
         <v>44560</v>
       </c>
-      <c r="X23" s="5"/>
-      <c r="Y23" s="5">
+      <c r="Y23" s="5"/>
+      <c r="Z23" s="5">
         <v>44560</v>
       </c>
-      <c r="Z23" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="AA23" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
+      </c>
+      <c r="AB23" s="4" t="s">
+        <v>220</v>
       </c>
     </row>
-    <row r="24" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
         <v>84</v>
       </c>
@@ -3034,44 +3226,47 @@
         <v>116</v>
       </c>
       <c r="O24" s="4" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="P24" s="4" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="Q24" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="R24" s="4">
+        <v>240</v>
+      </c>
+      <c r="R24" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="S24" s="4">
         <v>91.099239999999995</v>
       </c>
-      <c r="S24" s="4">
+      <c r="T24" s="4">
         <v>24.52702</v>
       </c>
-      <c r="T24" s="4" t="s">
+      <c r="U24" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U24" s="4" t="s">
+      <c r="V24" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V24" s="4" t="s">
+      <c r="W24" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W24" s="5">
+      <c r="X24" s="5">
         <v>39057</v>
       </c>
-      <c r="X24" s="5"/>
-      <c r="Y24" s="5">
+      <c r="Y24" s="5"/>
+      <c r="Z24" s="5">
         <v>43643</v>
       </c>
-      <c r="Z24" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="AA24" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
+      </c>
+      <c r="AB24" s="4" t="s">
+        <v>220</v>
       </c>
     </row>
-    <row r="25" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>86</v>
       </c>
@@ -3115,46 +3310,49 @@
         <v>116</v>
       </c>
       <c r="O25" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="P25" s="4" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="Q25" s="4" t="s">
-        <v>188</v>
-      </c>
-      <c r="R25" s="4">
+        <v>260</v>
+      </c>
+      <c r="R25" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="S25" s="4">
         <v>91.118949999999998</v>
       </c>
-      <c r="S25" s="4">
+      <c r="T25" s="4">
         <v>24.620080000000002</v>
       </c>
-      <c r="T25" s="4" t="s">
+      <c r="U25" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U25" s="4" t="s">
+      <c r="V25" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V25" s="4" t="s">
+      <c r="W25" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W25" s="5">
+      <c r="X25" s="5">
         <v>44376</v>
       </c>
-      <c r="X25" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="Y25" s="5">
+      <c r="Y25" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="Z25" s="5">
         <v>44376</v>
       </c>
-      <c r="Z25" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="AA25" s="4" t="s">
-        <v>225</v>
+        <v>223</v>
+      </c>
+      <c r="AB25" s="4" t="s">
+        <v>221</v>
       </c>
     </row>
-    <row r="26" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
         <v>92</v>
       </c>
@@ -3198,44 +3396,47 @@
         <v>116</v>
       </c>
       <c r="O26" s="4" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="P26" s="4" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="Q26" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="R26" s="4">
+        <v>241</v>
+      </c>
+      <c r="R26" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="S26" s="4">
         <v>91.086960000000005</v>
       </c>
-      <c r="S26" s="4">
+      <c r="T26" s="4">
         <v>24.449149999999999</v>
       </c>
-      <c r="T26" s="4" t="s">
+      <c r="U26" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U26" s="4" t="s">
+      <c r="V26" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V26" s="4" t="s">
+      <c r="W26" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W26" s="5">
+      <c r="X26" s="5">
         <v>41862</v>
       </c>
-      <c r="X26" s="5"/>
-      <c r="Y26" s="5">
+      <c r="Y26" s="5"/>
+      <c r="Z26" s="5">
         <v>43879</v>
       </c>
-      <c r="Z26" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="AA26" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
+      </c>
+      <c r="AB26" s="4" t="s">
+        <v>220</v>
       </c>
     </row>
-    <row r="27" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
         <v>96</v>
       </c>
@@ -3279,44 +3480,47 @@
         <v>116</v>
       </c>
       <c r="O27" s="4" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="P27" s="4" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="Q27" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="R27" s="4">
+        <v>261</v>
+      </c>
+      <c r="R27" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="S27" s="4">
         <v>91.067820999999995</v>
       </c>
-      <c r="S27" s="4">
+      <c r="T27" s="4">
         <v>24.469605999999999</v>
       </c>
-      <c r="T27" s="4" t="s">
+      <c r="U27" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U27" s="4" t="s">
+      <c r="V27" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V27" s="4" t="s">
+      <c r="W27" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W27" s="5">
+      <c r="X27" s="5">
         <v>45505</v>
       </c>
-      <c r="X27" s="5"/>
-      <c r="Y27" s="5">
+      <c r="Y27" s="5"/>
+      <c r="Z27" s="5">
         <v>45505</v>
       </c>
-      <c r="Z27" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="AA27" s="4" t="s">
-        <v>226</v>
+        <v>223</v>
+      </c>
+      <c r="AB27" s="4" t="s">
+        <v>222</v>
       </c>
     </row>
-    <row r="28" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
         <v>98</v>
       </c>
@@ -3360,44 +3564,47 @@
         <v>116</v>
       </c>
       <c r="O28" s="4" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="P28" s="4" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="Q28" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="R28" s="4">
+        <v>242</v>
+      </c>
+      <c r="R28" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="S28" s="4">
         <v>91.114959999999996</v>
       </c>
-      <c r="S28" s="4">
+      <c r="T28" s="4">
         <v>24.399149999999999</v>
       </c>
-      <c r="T28" s="4" t="s">
+      <c r="U28" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U28" s="4" t="s">
+      <c r="V28" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V28" s="4" t="s">
+      <c r="W28" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W28" s="5">
+      <c r="X28" s="5">
         <v>40110</v>
       </c>
-      <c r="X28" s="5"/>
-      <c r="Y28" s="5">
+      <c r="Y28" s="5"/>
+      <c r="Z28" s="5">
         <v>43642</v>
       </c>
-      <c r="Z28" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="AA28" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
+      </c>
+      <c r="AB28" s="4" t="s">
+        <v>220</v>
       </c>
     </row>
-    <row r="29" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>100</v>
       </c>
@@ -3441,44 +3648,47 @@
         <v>116</v>
       </c>
       <c r="O29" s="4" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="P29" s="4" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="Q29" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="R29" s="4">
+        <v>243</v>
+      </c>
+      <c r="R29" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="S29" s="4">
         <v>91.051150000000007</v>
       </c>
-      <c r="S29" s="4">
+      <c r="T29" s="4">
         <v>24.415769999999998</v>
       </c>
-      <c r="T29" s="4" t="s">
+      <c r="U29" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U29" s="4" t="s">
+      <c r="V29" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V29" s="4" t="s">
+      <c r="W29" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W29" s="5">
+      <c r="X29" s="5">
         <v>38714</v>
       </c>
-      <c r="X29" s="5"/>
-      <c r="Y29" s="5">
+      <c r="Y29" s="5"/>
+      <c r="Z29" s="5">
         <v>43614</v>
       </c>
-      <c r="Z29" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="AA29" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
+      </c>
+      <c r="AB29" s="4" t="s">
+        <v>220</v>
       </c>
     </row>
-    <row r="30" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>102</v>
       </c>
@@ -3522,44 +3732,47 @@
         <v>116</v>
       </c>
       <c r="O30" s="4" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="P30" s="4" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="Q30" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="R30" s="4">
+        <v>244</v>
+      </c>
+      <c r="R30" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="S30" s="4">
         <v>91.035638000000006</v>
       </c>
-      <c r="S30" s="4">
+      <c r="T30" s="4">
         <v>24.447555000000001</v>
       </c>
-      <c r="T30" s="4" t="s">
+      <c r="U30" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U30" s="4" t="s">
+      <c r="V30" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V30" s="4" t="s">
+      <c r="W30" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W30" s="5">
+      <c r="X30" s="5">
         <v>40543</v>
       </c>
-      <c r="X30" s="5"/>
-      <c r="Y30" s="5">
+      <c r="Y30" s="5"/>
+      <c r="Z30" s="5">
         <v>43877</v>
       </c>
-      <c r="Z30" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="AA30" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
+      </c>
+      <c r="AB30" s="4" t="s">
+        <v>220</v>
       </c>
     </row>
-    <row r="31" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>104</v>
       </c>
@@ -3603,44 +3816,47 @@
         <v>116</v>
       </c>
       <c r="O31" s="4" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="P31" s="4" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="Q31" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="R31" s="4">
+        <v>245</v>
+      </c>
+      <c r="R31" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="S31" s="4">
         <v>91.19247</v>
       </c>
-      <c r="S31" s="4">
+      <c r="T31" s="4">
         <v>24.432480000000002</v>
       </c>
-      <c r="T31" s="4" t="s">
+      <c r="U31" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U31" s="4" t="s">
+      <c r="V31" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V31" s="4" t="s">
+      <c r="W31" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W31" s="5">
+      <c r="X31" s="5">
         <v>44794</v>
       </c>
-      <c r="X31" s="5"/>
-      <c r="Y31" s="5">
+      <c r="Y31" s="5"/>
+      <c r="Z31" s="5">
         <v>44794</v>
-      </c>
-      <c r="Z31" s="4" t="s">
-        <v>227</v>
       </c>
       <c r="AA31" s="4" t="s">
         <v>223</v>
       </c>
+      <c r="AB31" s="4" t="s">
+        <v>219</v>
+      </c>
     </row>
-    <row r="32" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
         <v>106</v>
       </c>
@@ -3684,46 +3900,49 @@
         <v>116</v>
       </c>
       <c r="O32" s="4" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="P32" s="4" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="Q32" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="R32" s="4">
+        <v>246</v>
+      </c>
+      <c r="R32" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="S32" s="4">
         <v>91.050960000000003</v>
       </c>
-      <c r="S32" s="4">
+      <c r="T32" s="4">
         <v>24.409980000000001</v>
       </c>
-      <c r="T32" s="4" t="s">
+      <c r="U32" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U32" s="4" t="s">
+      <c r="V32" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V32" s="4" t="s">
+      <c r="W32" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W32" s="5">
+      <c r="X32" s="5">
         <v>44530</v>
       </c>
-      <c r="X32" s="5" t="s">
-        <v>222</v>
-      </c>
-      <c r="Y32" s="5">
+      <c r="Y32" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="Z32" s="5">
         <v>44530</v>
       </c>
-      <c r="Z32" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="AA32" s="4" t="s">
-        <v>225</v>
+        <v>223</v>
+      </c>
+      <c r="AB32" s="4" t="s">
+        <v>221</v>
       </c>
     </row>
-    <row r="33" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
         <v>108</v>
       </c>
@@ -3767,44 +3986,47 @@
         <v>116</v>
       </c>
       <c r="O33" s="4" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="P33" s="4" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="Q33" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="R33" s="4">
+        <v>247</v>
+      </c>
+      <c r="R33" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="S33" s="4">
         <v>91.054784999999995</v>
       </c>
-      <c r="S33" s="4">
+      <c r="T33" s="4">
         <v>24.416108000000001</v>
       </c>
-      <c r="T33" s="4" t="s">
+      <c r="U33" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U33" s="4" t="s">
+      <c r="V33" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V33" s="4" t="s">
+      <c r="W33" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W33" s="5">
+      <c r="X33" s="5">
         <v>44808</v>
       </c>
-      <c r="X33" s="5"/>
-      <c r="Y33" s="5">
+      <c r="Y33" s="5"/>
+      <c r="Z33" s="5">
         <v>44808</v>
-      </c>
-      <c r="Z33" s="4" t="s">
-        <v>227</v>
       </c>
       <c r="AA33" s="4" t="s">
         <v>223</v>
       </c>
+      <c r="AB33" s="4" t="s">
+        <v>219</v>
+      </c>
     </row>
-    <row r="34" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
         <v>110</v>
       </c>
@@ -3848,44 +4070,47 @@
         <v>116</v>
       </c>
       <c r="O34" s="4" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="P34" s="4" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="Q34" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="R34" s="4">
+        <v>248</v>
+      </c>
+      <c r="R34" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="S34" s="4">
         <v>91.148859999999999</v>
       </c>
-      <c r="S34" s="4">
+      <c r="T34" s="4">
         <v>24.42022</v>
       </c>
-      <c r="T34" s="4" t="s">
+      <c r="U34" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U34" s="4" t="s">
+      <c r="V34" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V34" s="4" t="s">
+      <c r="W34" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W34" s="5">
+      <c r="X34" s="5">
         <v>41999</v>
       </c>
-      <c r="X34" s="5"/>
-      <c r="Y34" s="5">
+      <c r="Y34" s="5"/>
+      <c r="Z34" s="5">
         <v>43901</v>
-      </c>
-      <c r="Z34" s="4" t="s">
-        <v>227</v>
       </c>
       <c r="AA34" s="4" t="s">
         <v>223</v>
       </c>
+      <c r="AB34" s="4" t="s">
+        <v>219</v>
+      </c>
     </row>
-    <row r="35" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>112</v>
       </c>
@@ -3929,44 +4154,47 @@
         <v>116</v>
       </c>
       <c r="O35" s="4" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="P35" s="4" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="Q35" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="R35" s="4">
+        <v>249</v>
+      </c>
+      <c r="R35" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="S35" s="4">
         <v>91.182230000000004</v>
       </c>
-      <c r="S35" s="4">
+      <c r="T35" s="4">
         <v>24.4633</v>
       </c>
-      <c r="T35" s="4" t="s">
+      <c r="U35" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="U35" s="4" t="s">
+      <c r="V35" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="V35" s="4" t="s">
+      <c r="W35" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="W35" s="5">
+      <c r="X35" s="5">
         <v>42023</v>
       </c>
-      <c r="X35" s="5"/>
-      <c r="Y35" s="5">
+      <c r="Y35" s="5"/>
+      <c r="Z35" s="5">
         <v>43868</v>
       </c>
-      <c r="Z35" s="4" t="s">
-        <v>227</v>
-      </c>
       <c r="AA35" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
+      </c>
+      <c r="AB35" s="4" t="s">
+        <v>220</v>
       </c>
     </row>
-    <row r="36" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
         <v>114</v>
       </c>
@@ -4010,41 +4238,44 @@
         <v>116</v>
       </c>
       <c r="O36" s="4" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="P36" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="Q36" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="R36" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="S36" s="4">
+        <v>91.056880000000007</v>
+      </c>
+      <c r="T36" s="4">
+        <v>24.410720000000001</v>
+      </c>
+      <c r="U36" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="V36" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="W36" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="X36" s="5">
+        <v>41727</v>
+      </c>
+      <c r="Y36" s="5"/>
+      <c r="Z36" s="5">
+        <v>43782</v>
+      </c>
+      <c r="AA36" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="AB36" s="4" t="s">
         <v>220</v>
-      </c>
-      <c r="Q36" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="R36" s="4">
-        <v>91.056880000000007</v>
-      </c>
-      <c r="S36" s="4">
-        <v>24.410720000000001</v>
-      </c>
-      <c r="T36" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="U36" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="V36" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="W36" s="5">
-        <v>41727</v>
-      </c>
-      <c r="X36" s="5"/>
-      <c r="Y36" s="5">
-        <v>43782</v>
-      </c>
-      <c r="Z36" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="AA36" s="4" t="s">
-        <v>224</v>
       </c>
     </row>
   </sheetData>

</xml_diff>